<commit_message>
Lengkapi workbook post-test: analisis waktu per butir dan audit kecukupan
Audit balik terhadap isi sel workbook menemukan satu celah: matriks waktu
per butir post-test ada di sheet Time Data ekspor resmi tetapi belum masuk
workbook, padahal workbook pre-test sudah memuatnya.

Menambah sheet 13 Analisis Waktu: waktu rata-rata per butir, matriks penuh
15x20 (218 sel), perbandingan waktu jawaban benar versus salah, dan dasar
forensik pengeluaran sesi QA tester -- 15 dari 20 butir dijawab dalam waktu
persis 1 detik.

Workbook post-test kini 13 sheet, 20 grafik. Audit kecukupan 60 pemeriksaan
seluruhnya lulus.
</commit_message>
<xml_diff>
--- a/LAPORAN_POSTTEST_DAN_PERBANDINGAN_CANVA.xlsx
+++ b/LAPORAN_POSTTEST_DAN_PERBANDINGAN_CANVA.xlsx
@@ -19,6 +19,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Dashboard Grafik" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 Data Mentah" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 Data Berpasangan" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13 Analisis Waktu" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -207,7 +208,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -357,6 +358,21 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1428,6 +1444,104 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart19.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Waktu rata-rata per butir post-test (detik)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'13 Analisis Waktu'!D5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'13 Analisis Waktu'!$A$6:$A$25</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'13 Analisis Waktu'!$D$6:$D$25</f>
+            </numRef>
+          </val>
+        </ser>
+        <dLbls>
+          <showVal val="1"/>
+        </dLbls>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Detik</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
@@ -1534,6 +1648,128 @@
                 </a:pPr>
                 <a:r>
                   <a:t>Jawaban benar (dari 20)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart20.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="12"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Waktu jawaban benar versus jawaban salah, per butir</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'13 Analisis Waktu'!I5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'13 Analisis Waktu'!$A$6:$A$25</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'13 Analisis Waktu'!$I$6:$I$25</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'13 Analisis Waktu'!J5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'13 Analisis Waktu'!$A$6:$A$25</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'13 Analisis Waktu'!$J$6:$J$25</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Detik</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -2794,6 +3030,55 @@
 </wsDr>
 </file>
 
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>26</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="9360000" cy="3240000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>45</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="9360000" cy="3240000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -3708,7 +3993,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F256"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -4943,7 +5228,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:V19"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
@@ -6761,7 +7046,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:L22"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
@@ -7361,6 +7646,2927 @@
     <mergeCell ref="A21:L21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:V118"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="76" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="6" max="6"/>
+    <col width="6" customWidth="1" min="7" max="7"/>
+    <col width="6" customWidth="1" min="8" max="8"/>
+    <col width="6" customWidth="1" min="9" max="9"/>
+    <col width="6" customWidth="1" min="10" max="10"/>
+    <col width="6" customWidth="1" min="11" max="11"/>
+    <col width="6" customWidth="1" min="12" max="12"/>
+    <col width="6" customWidth="1" min="13" max="13"/>
+    <col width="6" customWidth="1" min="14" max="14"/>
+    <col width="6" customWidth="1" min="15" max="15"/>
+    <col width="6" customWidth="1" min="16" max="16"/>
+    <col width="6" customWidth="1" min="17" max="17"/>
+    <col width="6" customWidth="1" min="18" max="18"/>
+    <col width="6" customWidth="1" min="19" max="19"/>
+    <col width="6" customWidth="1" min="20" max="20"/>
+    <col width="6" customWidth="1" min="21" max="21"/>
+    <col width="9" customWidth="1" min="22" max="22"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ANALISIS WAKTU POST-TEST — PER BUTIR DAN PER PESERTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Diambil utuh dari sheet Time Data ekspor resmi Wayground. Kolom Vincent ditampilkan terpisah pada bagian C sebagai bukti dasar pengeluaran sesi QA, tetapi tidak ikut dalam perhitungan rata-rata mana pun.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>A. WAKTU RATA-RATA PER BUTIR (15 sesi, Vincent dikeluarkan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Butir</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Pokok yang diuji</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Rata-rata
+Wayground</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Rata-rata
+hitung ulang</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Tercepat</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Terlama</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Penjawab</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>p</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>Waktu
+jawaban benar</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>Waktu
+jawaban salah</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>Selisih</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>Catatan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Kolaborasi real-time</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="D6" s="26" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>47</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="J6" s="6" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="K6" s="6" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="L6" s="8" t="inlineStr"/>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="33" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Asal usul Canva (Fusion Books)</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="D7" s="26" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>51</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="J7" s="6" t="n">
+        <v>26.8</v>
+      </c>
+      <c r="K7" s="6" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="L7" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Yang salah berpikir jauh lebih lama — butir membingungkan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="33" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Brand Kit</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="D8" s="26" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>66</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>36.2</v>
+      </c>
+      <c r="J8" s="6" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="K8" s="6" t="n">
+        <v>-13.4</v>
+      </c>
+      <c r="L8" s="8" t="inlineStr"/>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="33" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Hierarki visual — yang bertentangan</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="D9" s="26" t="n">
+        <v>33.5</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>67</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>36.8</v>
+      </c>
+      <c r="J9" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="K9" s="6" t="n">
+        <v>-17.8</v>
+      </c>
+      <c r="L9" s="8" t="inlineStr"/>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="33" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Harga paket Pro</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="D10" s="26" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="I10" s="6" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="J10" s="6" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="K10" s="6" t="n">
+        <v>-1</v>
+      </c>
+      <c r="L10" s="8" t="inlineStr"/>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="33" t="n">
+        <v>6</v>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Format ekspor PNG</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="D11" s="26" t="n">
+        <v>30.2</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>66</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="I11" s="6" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="J11" s="6" t="n">
+        <v>29.3</v>
+      </c>
+      <c r="K11" s="6" t="n">
+        <v>-1.2</v>
+      </c>
+      <c r="L11" s="8" t="inlineStr"/>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="33" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Pernyataan benar tentang Canva</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="D12" s="26" t="n">
+        <v>33.7</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>60</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="H12" s="6" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="I12" s="6" t="n">
+        <v>34</v>
+      </c>
+      <c r="J12" s="6" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="K12" s="6" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="L12" s="8" t="inlineStr"/>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="33" t="n">
+        <v>8</v>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Makna warna ungu liturgi</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="D13" s="26" t="n">
+        <v>26</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>64</v>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="H13" s="6" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="I13" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="J13" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K13" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L13" s="8" t="inlineStr"/>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="33" t="n">
+        <v>9</v>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>Format ekspor MP4</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="D14" s="26" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>38</v>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="H14" s="6" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="I14" s="6" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="J14" s="6" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="K14" s="6" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="L14" s="8" t="inlineStr"/>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="33" t="n">
+        <v>10</v>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Batas jumlah warna dan font</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>48</v>
+      </c>
+      <c r="D15" s="28" t="n">
+        <v>52.2</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="G15" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="H15" s="6" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="I15" s="6" t="n">
+        <v>53</v>
+      </c>
+      <c r="J15" s="6" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="K15" s="6" t="n">
+        <v>-4.5</v>
+      </c>
+      <c r="L15" s="8" t="inlineStr">
+        <is>
+          <t>Butir paling lama dibaca — redaksi opsinya panjang.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="33" t="n">
+        <v>11</v>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Menu panel kiri</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="D16" s="26" t="n">
+        <v>31.8</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="F16" s="6" t="n">
+        <v>76</v>
+      </c>
+      <c r="G16" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="H16" s="6" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="I16" s="6" t="n">
+        <v>29.4</v>
+      </c>
+      <c r="J16" s="6" t="n">
+        <v>33.8</v>
+      </c>
+      <c r="K16" s="6" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="L16" s="8" t="inlineStr"/>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="33" t="n">
+        <v>12</v>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Tiga pendiri Canva</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>33</v>
+      </c>
+      <c r="D17" s="26" t="n">
+        <v>35.6</v>
+      </c>
+      <c r="E17" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="F17" s="6" t="n">
+        <v>90</v>
+      </c>
+      <c r="G17" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="H17" s="6" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="I17" s="6" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="J17" s="6" t="n">
+        <v>36.3</v>
+      </c>
+      <c r="K17" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="L17" s="8" t="inlineStr"/>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="33" t="n">
+        <v>13</v>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>Eyedropper</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="D18" s="26" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="F18" s="6" t="n">
+        <v>94</v>
+      </c>
+      <c r="G18" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="H18" s="6" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="I18" s="6" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="J18" s="6" t="n">
+        <v>44</v>
+      </c>
+      <c r="K18" s="6" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="L18" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Yang salah berpikir jauh lebih lama — butir membingungkan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="33" t="n">
+        <v>14</v>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Ukuran Instagram Feed</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="D19" s="26" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="F19" s="6" t="n">
+        <v>42</v>
+      </c>
+      <c r="G19" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="H19" s="6" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="I19" s="6" t="n">
+        <v>23.9</v>
+      </c>
+      <c r="J19" s="6" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="K19" s="6" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="L19" s="8" t="inlineStr"/>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="33" t="n">
+        <v>15</v>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>Empat nilai berkarya</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>41</v>
+      </c>
+      <c r="D20" s="28" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="F20" s="6" t="n">
+        <v>132</v>
+      </c>
+      <c r="G20" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="H20" s="6" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="I20" s="6" t="n">
+        <v>55.3</v>
+      </c>
+      <c r="J20" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="K20" s="6" t="n">
+        <v>-32.3</v>
+      </c>
+      <c r="L20" s="8" t="inlineStr">
+        <is>
+          <t>Butir paling lama dibaca — redaksi opsinya panjang.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="33" t="n">
+        <v>16</v>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Urutan langkah template</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="D21" s="26" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="E21" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="F21" s="6" t="n">
+        <v>69</v>
+      </c>
+      <c r="G21" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="H21" s="6" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="I21" s="6" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="J21" s="6" t="n">
+        <v>37.4</v>
+      </c>
+      <c r="K21" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="L21" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Yang salah berpikir jauh lebih lama — butir membingungkan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="33" t="n">
+        <v>17</v>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>Komentar pada elemen</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="n">
+        <v>55</v>
+      </c>
+      <c r="D22" s="28" t="n">
+        <v>59.8</v>
+      </c>
+      <c r="E22" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="F22" s="6" t="n">
+        <v>343</v>
+      </c>
+      <c r="G22" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="H22" s="6" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="I22" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="J22" s="6" t="n">
+        <v>69.5</v>
+      </c>
+      <c r="K22" s="6" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="L22" s="8" t="inlineStr">
+        <is>
+          <t>Butir paling lama dibaca — redaksi opsinya panjang. Yang salah berpikir jauh lebih lama — butir membingungkan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="33" t="n">
+        <v>18</v>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>Etika AI</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="D23" s="26" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="E23" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>46</v>
+      </c>
+      <c r="G23" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="H23" s="6" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="I23" s="6" t="n">
+        <v>29.1</v>
+      </c>
+      <c r="J23" s="6" t="n">
+        <v>34.7</v>
+      </c>
+      <c r="K23" s="6" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="L23" s="8" t="inlineStr"/>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="33" t="n">
+        <v>19</v>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>Skema warna monokromatik</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="D24" s="26" t="n">
+        <v>33.9</v>
+      </c>
+      <c r="E24" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>70</v>
+      </c>
+      <c r="G24" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="H24" s="6" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="I24" s="6" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="J24" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="K24" s="6" t="n">
+        <v>-11.5</v>
+      </c>
+      <c r="L24" s="8" t="inlineStr"/>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="33" t="n">
+        <v>20</v>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Esensi tujuan pelatihan</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="D25" s="26" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="E25" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="F25" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="G25" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="H25" s="6" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="I25" s="6" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="J25" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K25" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L25" s="8" t="inlineStr"/>
+    </row>
+    <row r="66" ht="22" customHeight="1">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>B. MATRIKS WAKTU PENUH — 15 SESI x 20 BUTIR (detik)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="34" customHeight="1">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t>Nama</t>
+        </is>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t>Q5</t>
+        </is>
+      </c>
+      <c r="G67" s="4" t="inlineStr">
+        <is>
+          <t>Q6</t>
+        </is>
+      </c>
+      <c r="H67" s="4" t="inlineStr">
+        <is>
+          <t>Q7</t>
+        </is>
+      </c>
+      <c r="I67" s="4" t="inlineStr">
+        <is>
+          <t>Q8</t>
+        </is>
+      </c>
+      <c r="J67" s="4" t="inlineStr">
+        <is>
+          <t>Q9</t>
+        </is>
+      </c>
+      <c r="K67" s="4" t="inlineStr">
+        <is>
+          <t>Q10</t>
+        </is>
+      </c>
+      <c r="L67" s="4" t="inlineStr">
+        <is>
+          <t>Q11</t>
+        </is>
+      </c>
+      <c r="M67" s="4" t="inlineStr">
+        <is>
+          <t>Q12</t>
+        </is>
+      </c>
+      <c r="N67" s="4" t="inlineStr">
+        <is>
+          <t>Q13</t>
+        </is>
+      </c>
+      <c r="O67" s="4" t="inlineStr">
+        <is>
+          <t>Q14</t>
+        </is>
+      </c>
+      <c r="P67" s="4" t="inlineStr">
+        <is>
+          <t>Q15</t>
+        </is>
+      </c>
+      <c r="Q67" s="4" t="inlineStr">
+        <is>
+          <t>Q16</t>
+        </is>
+      </c>
+      <c r="R67" s="4" t="inlineStr">
+        <is>
+          <t>Q17</t>
+        </is>
+      </c>
+      <c r="S67" s="4" t="inlineStr">
+        <is>
+          <t>Q18</t>
+        </is>
+      </c>
+      <c r="T67" s="4" t="inlineStr">
+        <is>
+          <t>Q19</t>
+        </is>
+      </c>
+      <c r="U67" s="4" t="inlineStr">
+        <is>
+          <t>Q20</t>
+        </is>
+      </c>
+      <c r="V67" s="4" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="37" t="inlineStr">
+        <is>
+          <t>Agnes Nurak</t>
+        </is>
+      </c>
+      <c r="B68" s="56" t="n">
+        <v>32</v>
+      </c>
+      <c r="C68" s="56" t="n">
+        <v>17</v>
+      </c>
+      <c r="D68" s="56" t="n">
+        <v>22</v>
+      </c>
+      <c r="E68" s="56" t="n">
+        <v>31</v>
+      </c>
+      <c r="F68" s="56" t="n">
+        <v>17</v>
+      </c>
+      <c r="G68" s="56" t="n">
+        <v>32</v>
+      </c>
+      <c r="H68" s="56" t="n">
+        <v>31</v>
+      </c>
+      <c r="I68" s="56" t="n">
+        <v>29</v>
+      </c>
+      <c r="J68" s="56" t="n">
+        <v>24</v>
+      </c>
+      <c r="K68" s="56" t="n">
+        <v>39</v>
+      </c>
+      <c r="L68" s="56" t="n">
+        <v>23</v>
+      </c>
+      <c r="M68" s="56" t="n">
+        <v>13</v>
+      </c>
+      <c r="N68" s="56" t="n">
+        <v>21</v>
+      </c>
+      <c r="O68" s="56" t="n">
+        <v>16</v>
+      </c>
+      <c r="P68" s="56" t="n">
+        <v>32</v>
+      </c>
+      <c r="Q68" s="56" t="n">
+        <v>15</v>
+      </c>
+      <c r="R68" s="56" t="n">
+        <v>20</v>
+      </c>
+      <c r="S68" s="56" t="n">
+        <v>35</v>
+      </c>
+      <c r="T68" s="56" t="n">
+        <v>18</v>
+      </c>
+      <c r="U68" s="56" t="n">
+        <v>38</v>
+      </c>
+      <c r="V68" s="57" t="n">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="37" t="inlineStr">
+        <is>
+          <t>Mien</t>
+        </is>
+      </c>
+      <c r="B69" s="56" t="n">
+        <v>38</v>
+      </c>
+      <c r="C69" s="58" t="n">
+        <v>51</v>
+      </c>
+      <c r="D69" s="56" t="n">
+        <v>29</v>
+      </c>
+      <c r="E69" s="56" t="n">
+        <v>31</v>
+      </c>
+      <c r="F69" s="56" t="n">
+        <v>35</v>
+      </c>
+      <c r="G69" s="58" t="n">
+        <v>66</v>
+      </c>
+      <c r="H69" s="58" t="n">
+        <v>60</v>
+      </c>
+      <c r="I69" s="58" t="n">
+        <v>64</v>
+      </c>
+      <c r="J69" s="56" t="n">
+        <v>37</v>
+      </c>
+      <c r="K69" s="58" t="n">
+        <v>57</v>
+      </c>
+      <c r="L69" s="56" t="n">
+        <v>34</v>
+      </c>
+      <c r="M69" s="58" t="n">
+        <v>62</v>
+      </c>
+      <c r="N69" s="56" t="n">
+        <v>32</v>
+      </c>
+      <c r="O69" s="56" t="n">
+        <v>23</v>
+      </c>
+      <c r="P69" s="56" t="n">
+        <v>35</v>
+      </c>
+      <c r="Q69" s="56" t="n">
+        <v>33</v>
+      </c>
+      <c r="R69" s="56" t="n">
+        <v>22</v>
+      </c>
+      <c r="S69" s="58" t="n">
+        <v>46</v>
+      </c>
+      <c r="T69" s="58" t="n">
+        <v>53</v>
+      </c>
+      <c r="U69" s="58" t="n">
+        <v>50</v>
+      </c>
+      <c r="V69" s="57" t="n">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="37" t="inlineStr">
+        <is>
+          <t>LESLY MARCHRITH NUSALY</t>
+        </is>
+      </c>
+      <c r="B70" s="56" t="n">
+        <v>13</v>
+      </c>
+      <c r="C70" s="56" t="n">
+        <v>9</v>
+      </c>
+      <c r="D70" s="56" t="n">
+        <v>11</v>
+      </c>
+      <c r="E70" s="56" t="n">
+        <v>19</v>
+      </c>
+      <c r="F70" s="59" t="n">
+        <v>5</v>
+      </c>
+      <c r="G70" s="56" t="n">
+        <v>9</v>
+      </c>
+      <c r="H70" s="56" t="n">
+        <v>13</v>
+      </c>
+      <c r="I70" s="56" t="n">
+        <v>7</v>
+      </c>
+      <c r="J70" s="56" t="n">
+        <v>12</v>
+      </c>
+      <c r="K70" s="56" t="n">
+        <v>16</v>
+      </c>
+      <c r="L70" s="56" t="n">
+        <v>12</v>
+      </c>
+      <c r="M70" s="56" t="n">
+        <v>16</v>
+      </c>
+      <c r="N70" s="56" t="n">
+        <v>23</v>
+      </c>
+      <c r="O70" s="56" t="n">
+        <v>12</v>
+      </c>
+      <c r="P70" s="56" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q70" s="56" t="n">
+        <v>32</v>
+      </c>
+      <c r="R70" s="56" t="n">
+        <v>11</v>
+      </c>
+      <c r="S70" s="56" t="n">
+        <v>12</v>
+      </c>
+      <c r="T70" s="56" t="n">
+        <v>17</v>
+      </c>
+      <c r="U70" s="56" t="n">
+        <v>11</v>
+      </c>
+      <c r="V70" s="57" t="n">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="37" t="inlineStr">
+        <is>
+          <t>Gerarda Ina</t>
+        </is>
+      </c>
+      <c r="B71" s="56" t="n">
+        <v>31</v>
+      </c>
+      <c r="C71" s="56" t="n">
+        <v>40</v>
+      </c>
+      <c r="D71" s="58" t="n">
+        <v>66</v>
+      </c>
+      <c r="E71" s="58" t="n">
+        <v>67</v>
+      </c>
+      <c r="F71" s="56" t="n">
+        <v>6</v>
+      </c>
+      <c r="G71" s="58" t="n">
+        <v>45</v>
+      </c>
+      <c r="H71" s="58" t="n">
+        <v>49</v>
+      </c>
+      <c r="I71" s="56" t="n">
+        <v>14</v>
+      </c>
+      <c r="J71" s="56" t="n">
+        <v>38</v>
+      </c>
+      <c r="K71" s="58" t="n">
+        <v>66</v>
+      </c>
+      <c r="L71" s="56" t="n">
+        <v>27</v>
+      </c>
+      <c r="M71" s="56" t="n">
+        <v>31</v>
+      </c>
+      <c r="N71" s="56" t="n">
+        <v>19</v>
+      </c>
+      <c r="O71" s="56" t="n">
+        <v>42</v>
+      </c>
+      <c r="P71" s="58" t="n">
+        <v>132</v>
+      </c>
+      <c r="Q71" s="56" t="n">
+        <v>23</v>
+      </c>
+      <c r="R71" s="58" t="n">
+        <v>343</v>
+      </c>
+      <c r="S71" s="56" t="n">
+        <v>30</v>
+      </c>
+      <c r="T71" s="56" t="n">
+        <v>31</v>
+      </c>
+      <c r="U71" s="56" t="n">
+        <v>21</v>
+      </c>
+      <c r="V71" s="57" t="n">
+        <v>1121</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="37" t="inlineStr">
+        <is>
+          <t>Mirza Caroline</t>
+        </is>
+      </c>
+      <c r="B72" s="56" t="n">
+        <v>19</v>
+      </c>
+      <c r="C72" s="56" t="n">
+        <v>15</v>
+      </c>
+      <c r="D72" s="56" t="n">
+        <v>20</v>
+      </c>
+      <c r="E72" s="58" t="n">
+        <v>45</v>
+      </c>
+      <c r="F72" s="56" t="n">
+        <v>11</v>
+      </c>
+      <c r="G72" s="56" t="n">
+        <v>22</v>
+      </c>
+      <c r="H72" s="56" t="n">
+        <v>24</v>
+      </c>
+      <c r="I72" s="56" t="n">
+        <v>11</v>
+      </c>
+      <c r="J72" s="56" t="n">
+        <v>25</v>
+      </c>
+      <c r="K72" s="56" t="n">
+        <v>43</v>
+      </c>
+      <c r="L72" s="56" t="n">
+        <v>13</v>
+      </c>
+      <c r="M72" s="56" t="n">
+        <v>10</v>
+      </c>
+      <c r="N72" s="56" t="n">
+        <v>25</v>
+      </c>
+      <c r="O72" s="56" t="n">
+        <v>19</v>
+      </c>
+      <c r="P72" s="56" t="n">
+        <v>24</v>
+      </c>
+      <c r="Q72" s="56" t="n">
+        <v>21</v>
+      </c>
+      <c r="R72" s="56" t="n">
+        <v>17</v>
+      </c>
+      <c r="S72" s="56" t="n">
+        <v>26</v>
+      </c>
+      <c r="T72" s="56" t="n">
+        <v>18</v>
+      </c>
+      <c r="U72" s="56" t="n">
+        <v>14</v>
+      </c>
+      <c r="V72" s="57" t="n">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="37" t="inlineStr">
+        <is>
+          <t>wisye pangalila</t>
+        </is>
+      </c>
+      <c r="B73" s="56" t="n">
+        <v>18</v>
+      </c>
+      <c r="C73" s="56" t="n">
+        <v>17</v>
+      </c>
+      <c r="D73" s="56" t="n">
+        <v>23</v>
+      </c>
+      <c r="E73" s="56" t="n">
+        <v>29</v>
+      </c>
+      <c r="F73" s="56" t="n">
+        <v>12</v>
+      </c>
+      <c r="G73" s="56" t="n">
+        <v>9</v>
+      </c>
+      <c r="H73" s="56" t="n">
+        <v>16</v>
+      </c>
+      <c r="I73" s="56" t="n">
+        <v>27</v>
+      </c>
+      <c r="J73" s="56" t="n">
+        <v>15</v>
+      </c>
+      <c r="K73" s="56" t="n">
+        <v>41</v>
+      </c>
+      <c r="L73" s="56" t="n">
+        <v>37</v>
+      </c>
+      <c r="M73" s="56" t="n">
+        <v>28</v>
+      </c>
+      <c r="N73" s="56" t="n">
+        <v>14</v>
+      </c>
+      <c r="O73" s="56" t="n">
+        <v>14</v>
+      </c>
+      <c r="P73" s="58" t="n">
+        <v>47</v>
+      </c>
+      <c r="Q73" s="56" t="n">
+        <v>15</v>
+      </c>
+      <c r="R73" s="56" t="n">
+        <v>24</v>
+      </c>
+      <c r="S73" s="56" t="n">
+        <v>15</v>
+      </c>
+      <c r="T73" s="58" t="n">
+        <v>70</v>
+      </c>
+      <c r="U73" s="56" t="n">
+        <v>18</v>
+      </c>
+      <c r="V73" s="57" t="n">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="37" t="inlineStr">
+        <is>
+          <t>Yovita</t>
+        </is>
+      </c>
+      <c r="B74" s="58" t="n">
+        <v>47</v>
+      </c>
+      <c r="C74" s="56" t="n">
+        <v>26</v>
+      </c>
+      <c r="D74" s="56" t="n">
+        <v>28</v>
+      </c>
+      <c r="E74" s="58" t="n">
+        <v>62</v>
+      </c>
+      <c r="F74" s="56" t="n">
+        <v>20</v>
+      </c>
+      <c r="G74" s="56" t="n">
+        <v>24</v>
+      </c>
+      <c r="H74" s="56" t="n">
+        <v>26</v>
+      </c>
+      <c r="I74" s="58" t="n">
+        <v>57</v>
+      </c>
+      <c r="J74" s="56" t="n">
+        <v>32</v>
+      </c>
+      <c r="K74" s="58" t="n">
+        <v>100</v>
+      </c>
+      <c r="L74" s="56" t="n">
+        <v>39</v>
+      </c>
+      <c r="M74" s="56" t="n">
+        <v>42</v>
+      </c>
+      <c r="N74" s="56" t="n">
+        <v>32</v>
+      </c>
+      <c r="O74" s="56" t="n">
+        <v>30</v>
+      </c>
+      <c r="P74" s="58" t="n">
+        <v>69</v>
+      </c>
+      <c r="Q74" s="58" t="n">
+        <v>69</v>
+      </c>
+      <c r="R74" s="58" t="n">
+        <v>78</v>
+      </c>
+      <c r="S74" s="56" t="n">
+        <v>38</v>
+      </c>
+      <c r="T74" s="56" t="n">
+        <v>42</v>
+      </c>
+      <c r="U74" s="56" t="n">
+        <v>29</v>
+      </c>
+      <c r="V74" s="57" t="n">
+        <v>890</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="37" t="inlineStr">
+        <is>
+          <t>Netty Nusaly</t>
+        </is>
+      </c>
+      <c r="B75" s="56" t="n">
+        <v>12</v>
+      </c>
+      <c r="C75" s="56" t="n">
+        <v>9</v>
+      </c>
+      <c r="D75" s="56" t="n">
+        <v>23</v>
+      </c>
+      <c r="E75" s="56" t="n">
+        <v>21</v>
+      </c>
+      <c r="F75" s="56" t="n">
+        <v>16</v>
+      </c>
+      <c r="G75" s="56" t="n">
+        <v>29</v>
+      </c>
+      <c r="H75" s="56" t="n">
+        <v>41</v>
+      </c>
+      <c r="I75" s="56" t="n">
+        <v>22</v>
+      </c>
+      <c r="J75" s="56" t="n">
+        <v>15</v>
+      </c>
+      <c r="K75" s="56" t="n">
+        <v>31</v>
+      </c>
+      <c r="L75" s="56" t="n">
+        <v>37</v>
+      </c>
+      <c r="M75" s="56" t="n">
+        <v>33</v>
+      </c>
+      <c r="N75" s="56" t="n">
+        <v>24</v>
+      </c>
+      <c r="O75" s="56" t="n">
+        <v>35</v>
+      </c>
+      <c r="P75" s="56" t="n">
+        <v>26</v>
+      </c>
+      <c r="Q75" s="56" t="n">
+        <v>28</v>
+      </c>
+      <c r="R75" s="56" t="n">
+        <v>27</v>
+      </c>
+      <c r="S75" s="56" t="n">
+        <v>32</v>
+      </c>
+      <c r="T75" s="56" t="n">
+        <v>33</v>
+      </c>
+      <c r="U75" s="56" t="n">
+        <v>26</v>
+      </c>
+      <c r="V75" s="57" t="n">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="37" t="inlineStr">
+        <is>
+          <t>Ivo Emelia</t>
+        </is>
+      </c>
+      <c r="B76" s="56" t="n">
+        <v>43</v>
+      </c>
+      <c r="C76" s="56" t="n">
+        <v>28</v>
+      </c>
+      <c r="D76" s="56" t="n">
+        <v>13</v>
+      </c>
+      <c r="E76" s="56" t="n">
+        <v>26</v>
+      </c>
+      <c r="F76" s="56" t="n">
+        <v>7</v>
+      </c>
+      <c r="G76" s="56" t="n">
+        <v>19</v>
+      </c>
+      <c r="H76" s="56" t="n">
+        <v>25</v>
+      </c>
+      <c r="I76" s="56" t="n">
+        <v>16</v>
+      </c>
+      <c r="J76" s="56" t="n">
+        <v>13</v>
+      </c>
+      <c r="K76" s="56" t="n">
+        <v>31</v>
+      </c>
+      <c r="L76" s="56" t="n">
+        <v>14</v>
+      </c>
+      <c r="M76" s="56" t="n">
+        <v>39</v>
+      </c>
+      <c r="N76" s="56" t="n">
+        <v>19</v>
+      </c>
+      <c r="O76" s="56" t="n">
+        <v>35</v>
+      </c>
+      <c r="P76" s="58" t="n">
+        <v>57</v>
+      </c>
+      <c r="Q76" s="56" t="n">
+        <v>41</v>
+      </c>
+      <c r="R76" s="56" t="n">
+        <v>29</v>
+      </c>
+      <c r="S76" s="56" t="n">
+        <v>31</v>
+      </c>
+      <c r="T76" s="56" t="n">
+        <v>31</v>
+      </c>
+      <c r="U76" s="56" t="n">
+        <v>26</v>
+      </c>
+      <c r="V76" s="57" t="n">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="37" t="inlineStr">
+        <is>
+          <t>Marsia Sairina</t>
+        </is>
+      </c>
+      <c r="B77" s="56" t="n">
+        <v>21</v>
+      </c>
+      <c r="C77" s="56" t="n">
+        <v>20</v>
+      </c>
+      <c r="D77" s="56" t="n">
+        <v>22</v>
+      </c>
+      <c r="E77" s="56" t="n">
+        <v>28</v>
+      </c>
+      <c r="F77" s="56" t="n">
+        <v>16</v>
+      </c>
+      <c r="G77" s="56" t="n">
+        <v>23</v>
+      </c>
+      <c r="H77" s="56" t="n">
+        <v>31</v>
+      </c>
+      <c r="I77" s="56" t="n">
+        <v>22</v>
+      </c>
+      <c r="J77" s="56" t="n">
+        <v>21</v>
+      </c>
+      <c r="K77" s="58" t="n">
+        <v>56</v>
+      </c>
+      <c r="L77" s="56" t="n">
+        <v>38</v>
+      </c>
+      <c r="M77" s="56" t="n">
+        <v>28</v>
+      </c>
+      <c r="N77" s="56" t="n">
+        <v>33</v>
+      </c>
+      <c r="O77" s="56" t="n">
+        <v>28</v>
+      </c>
+      <c r="P77" s="56" t="n">
+        <v>26</v>
+      </c>
+      <c r="Q77" s="56" t="n">
+        <v>37</v>
+      </c>
+      <c r="R77" s="56" t="n">
+        <v>27</v>
+      </c>
+      <c r="S77" s="56" t="n">
+        <v>43</v>
+      </c>
+      <c r="T77" s="56" t="n">
+        <v>26</v>
+      </c>
+      <c r="U77" s="56" t="n">
+        <v>26</v>
+      </c>
+      <c r="V77" s="57" t="n">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="37" t="inlineStr">
+        <is>
+          <t>Silvya Runturambi</t>
+        </is>
+      </c>
+      <c r="B78" s="56" t="n">
+        <v>12</v>
+      </c>
+      <c r="C78" s="56" t="n">
+        <v>19</v>
+      </c>
+      <c r="D78" s="58" t="n">
+        <v>47</v>
+      </c>
+      <c r="E78" s="56" t="n">
+        <v>10</v>
+      </c>
+      <c r="F78" s="56" t="n">
+        <v>24</v>
+      </c>
+      <c r="G78" s="58" t="n">
+        <v>54</v>
+      </c>
+      <c r="H78" s="58" t="n">
+        <v>55</v>
+      </c>
+      <c r="I78" s="56" t="n">
+        <v>17</v>
+      </c>
+      <c r="J78" s="56" t="n">
+        <v>38</v>
+      </c>
+      <c r="K78" s="58" t="n">
+        <v>94</v>
+      </c>
+      <c r="L78" s="58" t="n">
+        <v>76</v>
+      </c>
+      <c r="M78" s="58" t="n">
+        <v>90</v>
+      </c>
+      <c r="N78" s="58" t="n">
+        <v>94</v>
+      </c>
+      <c r="O78" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P78" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q78" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R78" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S78" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="T78" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="U78" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="V78" s="57" t="n">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="37" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="B79" s="56" t="n">
+        <v>8</v>
+      </c>
+      <c r="C79" s="56" t="n">
+        <v>11</v>
+      </c>
+      <c r="D79" s="56" t="n">
+        <v>24</v>
+      </c>
+      <c r="E79" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F79" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G79" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H79" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I79" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J79" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K79" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L79" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M79" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N79" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O79" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P79" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q79" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R79" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S79" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="T79" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="U79" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="V79" s="57" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="37" t="inlineStr">
+        <is>
+          <t>Ivonne runturambi</t>
+        </is>
+      </c>
+      <c r="B80" s="56" t="n">
+        <v>21</v>
+      </c>
+      <c r="C80" s="56" t="n">
+        <v>20</v>
+      </c>
+      <c r="D80" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E80" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F80" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G80" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H80" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I80" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J80" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K80" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L80" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M80" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N80" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O80" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P80" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q80" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R80" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S80" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="T80" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="U80" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="V80" s="57" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="37" t="inlineStr">
+        <is>
+          <t>Tintin tityn</t>
+        </is>
+      </c>
+      <c r="B81" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C81" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D81" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E81" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F81" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G81" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H81" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I81" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J81" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K81" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L81" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M81" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N81" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O81" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P81" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q81" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R81" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S81" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="T81" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="U81" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="V81" s="57" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="37" t="inlineStr">
+        <is>
+          <t>Yovita*</t>
+        </is>
+      </c>
+      <c r="B82" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C82" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D82" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E82" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F82" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G82" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H82" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I82" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J82" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K82" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L82" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M82" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N82" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O82" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P82" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q82" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="R82" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S82" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="T82" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="U82" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="V82" s="57" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" ht="32" customHeight="1">
+      <c r="A84" s="15" t="inlineStr">
+        <is>
+          <t>Merah = 5 detik atau kurang (terlalu cepat untuk membaca soal) · hijau = wajar · kuning = 45 detik atau lebih · abu-abu = butir tidak dijawab. Total 218 sel waktu terisi dari 300 sel yang mungkin; sisanya adalah butir yang memang tidak dijawab pada sesi terputus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="22" customHeight="1">
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t>C. DASAR FORENSIK PENGELUARAN SESI QA TESTER (VINCENT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="34" customHeight="1">
+      <c r="A87" s="4" t="inlineStr">
+        <is>
+          <t>Butir</t>
+        </is>
+      </c>
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t>Waktu Vincent
+(detik)</t>
+        </is>
+      </c>
+      <c r="C87" s="4" t="inlineStr">
+        <is>
+          <t>Rata-rata
+15 peserta</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="inlineStr">
+        <is>
+          <t>Selisih</t>
+        </is>
+      </c>
+      <c r="E87" s="4" t="inlineStr">
+        <is>
+          <t>Penilaian</t>
+        </is>
+      </c>
+      <c r="F87" s="4" t="inlineStr"/>
+      <c r="G87" s="4" t="inlineStr"/>
+      <c r="H87" s="4" t="inlineStr"/>
+      <c r="I87" s="4" t="inlineStr"/>
+      <c r="J87" s="4" t="inlineStr"/>
+      <c r="K87" s="4" t="inlineStr"/>
+      <c r="L87" s="4" t="inlineStr"/>
+    </row>
+    <row r="88" ht="18" customHeight="1">
+      <c r="A88" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="B88" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="C88" s="6" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="D88" s="6" t="n">
+        <v>-23.2</v>
+      </c>
+      <c r="E88" s="8" t="inlineStr">
+        <is>
+          <t>Satu detik — mustahil untuk membaca soal beserta empat opsinya.</t>
+        </is>
+      </c>
+      <c r="F88" s="9" t="n"/>
+      <c r="G88" s="9" t="n"/>
+      <c r="H88" s="9" t="n"/>
+      <c r="I88" s="9" t="n"/>
+      <c r="J88" s="9" t="n"/>
+      <c r="K88" s="9" t="n"/>
+      <c r="L88" s="10" t="n"/>
+    </row>
+    <row r="89" ht="18" customHeight="1">
+      <c r="A89" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="B89" s="17" t="n">
+        <v>64</v>
+      </c>
+      <c r="C89" s="6" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="D89" s="6" t="n">
+        <v>42.3</v>
+      </c>
+      <c r="E89" s="8" t="inlineStr">
+        <is>
+          <t>Wajar.</t>
+        </is>
+      </c>
+      <c r="F89" s="9" t="n"/>
+      <c r="G89" s="9" t="n"/>
+      <c r="H89" s="9" t="n"/>
+      <c r="I89" s="9" t="n"/>
+      <c r="J89" s="9" t="n"/>
+      <c r="K89" s="9" t="n"/>
+      <c r="L89" s="10" t="n"/>
+    </row>
+    <row r="90" ht="18" customHeight="1">
+      <c r="A90" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="B90" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="C90" s="6" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="D90" s="6" t="n">
+        <v>-26.3</v>
+      </c>
+      <c r="E90" s="8" t="inlineStr">
+        <is>
+          <t>Satu detik — mustahil untuk membaca soal beserta empat opsinya.</t>
+        </is>
+      </c>
+      <c r="F90" s="9" t="n"/>
+      <c r="G90" s="9" t="n"/>
+      <c r="H90" s="9" t="n"/>
+      <c r="I90" s="9" t="n"/>
+      <c r="J90" s="9" t="n"/>
+      <c r="K90" s="9" t="n"/>
+      <c r="L90" s="10" t="n"/>
+    </row>
+    <row r="91" ht="18" customHeight="1">
+      <c r="A91" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="B91" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="C91" s="6" t="n">
+        <v>33.5</v>
+      </c>
+      <c r="D91" s="6" t="n">
+        <v>-32.5</v>
+      </c>
+      <c r="E91" s="8" t="inlineStr">
+        <is>
+          <t>Satu detik — mustahil untuk membaca soal beserta empat opsinya.</t>
+        </is>
+      </c>
+      <c r="F91" s="9" t="n"/>
+      <c r="G91" s="9" t="n"/>
+      <c r="H91" s="9" t="n"/>
+      <c r="I91" s="9" t="n"/>
+      <c r="J91" s="9" t="n"/>
+      <c r="K91" s="9" t="n"/>
+      <c r="L91" s="10" t="n"/>
+    </row>
+    <row r="92" ht="18" customHeight="1">
+      <c r="A92" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="B92" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="C92" s="6" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="D92" s="6" t="n">
+        <v>-14.4</v>
+      </c>
+      <c r="E92" s="8" t="inlineStr">
+        <is>
+          <t>Satu detik — mustahil untuk membaca soal beserta empat opsinya.</t>
+        </is>
+      </c>
+      <c r="F92" s="9" t="n"/>
+      <c r="G92" s="9" t="n"/>
+      <c r="H92" s="9" t="n"/>
+      <c r="I92" s="9" t="n"/>
+      <c r="J92" s="9" t="n"/>
+      <c r="K92" s="9" t="n"/>
+      <c r="L92" s="10" t="n"/>
+    </row>
+    <row r="93" ht="18" customHeight="1">
+      <c r="A93" s="24" t="n">
+        <v>6</v>
+      </c>
+      <c r="B93" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="C93" s="6" t="n">
+        <v>30.2</v>
+      </c>
+      <c r="D93" s="6" t="n">
+        <v>-29.2</v>
+      </c>
+      <c r="E93" s="8" t="inlineStr">
+        <is>
+          <t>Satu detik — mustahil untuk membaca soal beserta empat opsinya.</t>
+        </is>
+      </c>
+      <c r="F93" s="9" t="n"/>
+      <c r="G93" s="9" t="n"/>
+      <c r="H93" s="9" t="n"/>
+      <c r="I93" s="9" t="n"/>
+      <c r="J93" s="9" t="n"/>
+      <c r="K93" s="9" t="n"/>
+      <c r="L93" s="10" t="n"/>
+    </row>
+    <row r="94" ht="18" customHeight="1">
+      <c r="A94" s="24" t="n">
+        <v>7</v>
+      </c>
+      <c r="B94" s="28" t="n">
+        <v>3</v>
+      </c>
+      <c r="C94" s="6" t="n">
+        <v>33.7</v>
+      </c>
+      <c r="D94" s="6" t="n">
+        <v>-30.7</v>
+      </c>
+      <c r="E94" s="8" t="inlineStr">
+        <is>
+          <t>Di bawah 5 detik; masih terlalu cepat untuk dibaca.</t>
+        </is>
+      </c>
+      <c r="F94" s="9" t="n"/>
+      <c r="G94" s="9" t="n"/>
+      <c r="H94" s="9" t="n"/>
+      <c r="I94" s="9" t="n"/>
+      <c r="J94" s="9" t="n"/>
+      <c r="K94" s="9" t="n"/>
+      <c r="L94" s="10" t="n"/>
+    </row>
+    <row r="95" ht="18" customHeight="1">
+      <c r="A95" s="24" t="n">
+        <v>8</v>
+      </c>
+      <c r="B95" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="C95" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="D95" s="6" t="n">
+        <v>-25</v>
+      </c>
+      <c r="E95" s="8" t="inlineStr">
+        <is>
+          <t>Satu detik — mustahil untuk membaca soal beserta empat opsinya.</t>
+        </is>
+      </c>
+      <c r="F95" s="9" t="n"/>
+      <c r="G95" s="9" t="n"/>
+      <c r="H95" s="9" t="n"/>
+      <c r="I95" s="9" t="n"/>
+      <c r="J95" s="9" t="n"/>
+      <c r="K95" s="9" t="n"/>
+      <c r="L95" s="10" t="n"/>
+    </row>
+    <row r="96" ht="18" customHeight="1">
+      <c r="A96" s="24" t="n">
+        <v>9</v>
+      </c>
+      <c r="B96" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="C96" s="6" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="D96" s="6" t="n">
+        <v>-23.5</v>
+      </c>
+      <c r="E96" s="8" t="inlineStr">
+        <is>
+          <t>Satu detik — mustahil untuk membaca soal beserta empat opsinya.</t>
+        </is>
+      </c>
+      <c r="F96" s="9" t="n"/>
+      <c r="G96" s="9" t="n"/>
+      <c r="H96" s="9" t="n"/>
+      <c r="I96" s="9" t="n"/>
+      <c r="J96" s="9" t="n"/>
+      <c r="K96" s="9" t="n"/>
+      <c r="L96" s="10" t="n"/>
+    </row>
+    <row r="97" ht="18" customHeight="1">
+      <c r="A97" s="24" t="n">
+        <v>10</v>
+      </c>
+      <c r="B97" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="C97" s="6" t="n">
+        <v>52.2</v>
+      </c>
+      <c r="D97" s="6" t="n">
+        <v>-51.2</v>
+      </c>
+      <c r="E97" s="8" t="inlineStr">
+        <is>
+          <t>Satu detik — mustahil untuk membaca soal beserta empat opsinya.</t>
+        </is>
+      </c>
+      <c r="F97" s="9" t="n"/>
+      <c r="G97" s="9" t="n"/>
+      <c r="H97" s="9" t="n"/>
+      <c r="I97" s="9" t="n"/>
+      <c r="J97" s="9" t="n"/>
+      <c r="K97" s="9" t="n"/>
+      <c r="L97" s="10" t="n"/>
+    </row>
+    <row r="98" ht="18" customHeight="1">
+      <c r="A98" s="24" t="n">
+        <v>11</v>
+      </c>
+      <c r="B98" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="C98" s="6" t="n">
+        <v>31.8</v>
+      </c>
+      <c r="D98" s="6" t="n">
+        <v>-30.8</v>
+      </c>
+      <c r="E98" s="8" t="inlineStr">
+        <is>
+          <t>Satu detik — mustahil untuk membaca soal beserta empat opsinya.</t>
+        </is>
+      </c>
+      <c r="F98" s="9" t="n"/>
+      <c r="G98" s="9" t="n"/>
+      <c r="H98" s="9" t="n"/>
+      <c r="I98" s="9" t="n"/>
+      <c r="J98" s="9" t="n"/>
+      <c r="K98" s="9" t="n"/>
+      <c r="L98" s="10" t="n"/>
+    </row>
+    <row r="99" ht="18" customHeight="1">
+      <c r="A99" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="B99" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="C99" s="6" t="n">
+        <v>35.6</v>
+      </c>
+      <c r="D99" s="6" t="n">
+        <v>-34.6</v>
+      </c>
+      <c r="E99" s="8" t="inlineStr">
+        <is>
+          <t>Satu detik — mustahil untuk membaca soal beserta empat opsinya.</t>
+        </is>
+      </c>
+      <c r="F99" s="9" t="n"/>
+      <c r="G99" s="9" t="n"/>
+      <c r="H99" s="9" t="n"/>
+      <c r="I99" s="9" t="n"/>
+      <c r="J99" s="9" t="n"/>
+      <c r="K99" s="9" t="n"/>
+      <c r="L99" s="10" t="n"/>
+    </row>
+    <row r="100" ht="18" customHeight="1">
+      <c r="A100" s="24" t="n">
+        <v>13</v>
+      </c>
+      <c r="B100" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="C100" s="6" t="n">
+        <v>30.5</v>
+      </c>
+      <c r="D100" s="6" t="n">
+        <v>-29.5</v>
+      </c>
+      <c r="E100" s="8" t="inlineStr">
+        <is>
+          <t>Satu detik — mustahil untuk membaca soal beserta empat opsinya.</t>
+        </is>
+      </c>
+      <c r="F100" s="9" t="n"/>
+      <c r="G100" s="9" t="n"/>
+      <c r="H100" s="9" t="n"/>
+      <c r="I100" s="9" t="n"/>
+      <c r="J100" s="9" t="n"/>
+      <c r="K100" s="9" t="n"/>
+      <c r="L100" s="10" t="n"/>
+    </row>
+    <row r="101" ht="18" customHeight="1">
+      <c r="A101" s="24" t="n">
+        <v>14</v>
+      </c>
+      <c r="B101" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="C101" s="6" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="D101" s="6" t="n">
+        <v>-24.4</v>
+      </c>
+      <c r="E101" s="8" t="inlineStr">
+        <is>
+          <t>Satu detik — mustahil untuk membaca soal beserta empat opsinya.</t>
+        </is>
+      </c>
+      <c r="F101" s="9" t="n"/>
+      <c r="G101" s="9" t="n"/>
+      <c r="H101" s="9" t="n"/>
+      <c r="I101" s="9" t="n"/>
+      <c r="J101" s="9" t="n"/>
+      <c r="K101" s="9" t="n"/>
+      <c r="L101" s="10" t="n"/>
+    </row>
+    <row r="102" ht="18" customHeight="1">
+      <c r="A102" s="24" t="n">
+        <v>15</v>
+      </c>
+      <c r="B102" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="C102" s="6" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="D102" s="6" t="n">
+        <v>-44.6</v>
+      </c>
+      <c r="E102" s="8" t="inlineStr">
+        <is>
+          <t>Satu detik — mustahil untuk membaca soal beserta empat opsinya.</t>
+        </is>
+      </c>
+      <c r="F102" s="9" t="n"/>
+      <c r="G102" s="9" t="n"/>
+      <c r="H102" s="9" t="n"/>
+      <c r="I102" s="9" t="n"/>
+      <c r="J102" s="9" t="n"/>
+      <c r="K102" s="9" t="n"/>
+      <c r="L102" s="10" t="n"/>
+    </row>
+    <row r="103" ht="18" customHeight="1">
+      <c r="A103" s="24" t="n">
+        <v>16</v>
+      </c>
+      <c r="B103" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="C103" s="6" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="D103" s="6" t="n">
+        <v>-30.4</v>
+      </c>
+      <c r="E103" s="8" t="inlineStr">
+        <is>
+          <t>Satu detik — mustahil untuk membaca soal beserta empat opsinya.</t>
+        </is>
+      </c>
+      <c r="F103" s="9" t="n"/>
+      <c r="G103" s="9" t="n"/>
+      <c r="H103" s="9" t="n"/>
+      <c r="I103" s="9" t="n"/>
+      <c r="J103" s="9" t="n"/>
+      <c r="K103" s="9" t="n"/>
+      <c r="L103" s="10" t="n"/>
+    </row>
+    <row r="104" ht="18" customHeight="1">
+      <c r="A104" s="24" t="n">
+        <v>17</v>
+      </c>
+      <c r="B104" s="28" t="n">
+        <v>2</v>
+      </c>
+      <c r="C104" s="6" t="n">
+        <v>59.8</v>
+      </c>
+      <c r="D104" s="6" t="n">
+        <v>-57.8</v>
+      </c>
+      <c r="E104" s="8" t="inlineStr">
+        <is>
+          <t>Di bawah 5 detik; masih terlalu cepat untuk dibaca.</t>
+        </is>
+      </c>
+      <c r="F104" s="9" t="n"/>
+      <c r="G104" s="9" t="n"/>
+      <c r="H104" s="9" t="n"/>
+      <c r="I104" s="9" t="n"/>
+      <c r="J104" s="9" t="n"/>
+      <c r="K104" s="9" t="n"/>
+      <c r="L104" s="10" t="n"/>
+    </row>
+    <row r="105" ht="18" customHeight="1">
+      <c r="A105" s="24" t="n">
+        <v>18</v>
+      </c>
+      <c r="B105" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="C105" s="6" t="n">
+        <v>30.8</v>
+      </c>
+      <c r="D105" s="6" t="n">
+        <v>-29.8</v>
+      </c>
+      <c r="E105" s="8" t="inlineStr">
+        <is>
+          <t>Satu detik — mustahil untuk membaca soal beserta empat opsinya.</t>
+        </is>
+      </c>
+      <c r="F105" s="9" t="n"/>
+      <c r="G105" s="9" t="n"/>
+      <c r="H105" s="9" t="n"/>
+      <c r="I105" s="9" t="n"/>
+      <c r="J105" s="9" t="n"/>
+      <c r="K105" s="9" t="n"/>
+      <c r="L105" s="10" t="n"/>
+    </row>
+    <row r="106" ht="18" customHeight="1">
+      <c r="A106" s="24" t="n">
+        <v>19</v>
+      </c>
+      <c r="B106" s="28" t="n">
+        <v>2</v>
+      </c>
+      <c r="C106" s="6" t="n">
+        <v>33.9</v>
+      </c>
+      <c r="D106" s="6" t="n">
+        <v>-31.9</v>
+      </c>
+      <c r="E106" s="8" t="inlineStr">
+        <is>
+          <t>Di bawah 5 detik; masih terlalu cepat untuk dibaca.</t>
+        </is>
+      </c>
+      <c r="F106" s="9" t="n"/>
+      <c r="G106" s="9" t="n"/>
+      <c r="H106" s="9" t="n"/>
+      <c r="I106" s="9" t="n"/>
+      <c r="J106" s="9" t="n"/>
+      <c r="K106" s="9" t="n"/>
+      <c r="L106" s="10" t="n"/>
+    </row>
+    <row r="107" ht="18" customHeight="1">
+      <c r="A107" s="24" t="n">
+        <v>20</v>
+      </c>
+      <c r="B107" s="28" t="n">
+        <v>2</v>
+      </c>
+      <c r="C107" s="6" t="n">
+        <v>25.9</v>
+      </c>
+      <c r="D107" s="6" t="n">
+        <v>-23.9</v>
+      </c>
+      <c r="E107" s="8" t="inlineStr">
+        <is>
+          <t>Di bawah 5 detik; masih terlalu cepat untuk dibaca.</t>
+        </is>
+      </c>
+      <c r="F107" s="9" t="n"/>
+      <c r="G107" s="9" t="n"/>
+      <c r="H107" s="9" t="n"/>
+      <c r="I107" s="9" t="n"/>
+      <c r="J107" s="9" t="n"/>
+      <c r="K107" s="9" t="n"/>
+      <c r="L107" s="10" t="n"/>
+    </row>
+    <row r="109" ht="40" customHeight="1">
+      <c r="A109" s="15" t="inlineStr">
+        <is>
+          <t>Dari 20 butir, 15 dijawab Vincent dalam waktu persis 1 detik. Membaca satu butir post-test beserta keempat opsinya membutuhkan sekurang-kurangnya beberapa detik; rata-rata 15 peserta lain adalah 31.7 detik per butir. Pola satu detik berulang adalah tanda penelusuran otomatis atau klik cepat untuk menguji jalannya kuis, bukan pengerjaan soal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="40" customHeight="1">
+      <c r="A110" s="15" t="inlineStr">
+        <is>
+          <t>Waktu total sesi Vincent 1 menit 28 detik untuk 20 butir, sementara rata-rata sesi tuntas peserta lain adalah 10 menit 18 detik.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="40" customHeight="1">
+      <c r="A111" s="15" t="inlineStr">
+        <is>
+          <t>Vincent juga tidak muncul pada daftar 37 peserta pre-test, sehingga tidak dapat masuk analisis berpasangan dalam keadaan apa pun.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="40" customHeight="1">
+      <c r="A112" s="15" t="inlineStr">
+        <is>
+          <t>Atas ketiga dasar itu sesi ini dikeluarkan dari seluruh perhitungan. Dampaknya terhadap angka agregat kecil dan dilaporkan penuh pada sheet 09 Metodologi bagian C: rata-rata turun 0,19 butir, akurasi turun 0,96 poin persen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="22" customHeight="1">
+      <c r="A114" s="3" t="inlineStr">
+        <is>
+          <t>D. TEMUAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="40" customHeight="1">
+      <c r="A115" s="15" t="inlineStr">
+        <is>
+          <t>Rata-rata waktu per butir 31.7 detik, dengan rentang 5 sampai 343 detik. Sebagai pembanding, pre-test yang dijalankan live mencatat rata-rata 17-18 detik per butir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="40" customHeight="1">
+      <c r="A116" s="15" t="inlineStr">
+        <is>
+          <t>Jawaban benar rata-rata memakan 30.5 detik, jawaban salah 34.2 detik — selisih 3.7 detik. Peserta yang menjawab salah justru berpikir sedikit lebih lama, sehingga tidak ada bukti kesalahan disebabkan oleh terburu-buru.</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="40" customHeight="1">
+      <c r="A117" s="15" t="inlineStr">
+        <is>
+          <t>Meskipun kuis dibuka tiga hari, tidak ada sesi tuntas yang memakai waktu ekstrem: yang tercepat 4 menit 28 detik dan yang terlama 18 menit 41 detik. Artinya peserta mengerjakan dalam satu duduk, bukan mencicil selama tiga hari.</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="40" customHeight="1">
+      <c r="A118" s="15" t="inlineStr">
+        <is>
+          <t>Perlu dicatat bahwa waktu tercatat hanya menghitung durasi butir terbuka di layar. Dalam mode take-home, peserta dapat membuka materi pada perangkat lain tanpa terekam sebagai waktu pengerjaan. Karena itu waktu yang wajar pada tabel ini bukan bukti bahwa pengerjaan dilakukan tanpa membuka materi.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="35">
+    <mergeCell ref="E96:L96"/>
+    <mergeCell ref="E106:L106"/>
+    <mergeCell ref="A84:L84"/>
+    <mergeCell ref="A66:L66"/>
+    <mergeCell ref="A118:L118"/>
+    <mergeCell ref="E98:L98"/>
+    <mergeCell ref="E92:L92"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A86:L86"/>
+    <mergeCell ref="E88:L88"/>
+    <mergeCell ref="E107:L107"/>
+    <mergeCell ref="A116:L116"/>
+    <mergeCell ref="E94:L94"/>
+    <mergeCell ref="E103:L103"/>
+    <mergeCell ref="A109:L109"/>
+    <mergeCell ref="A4:L4"/>
+    <mergeCell ref="A112:L112"/>
+    <mergeCell ref="E90:L90"/>
+    <mergeCell ref="E105:L105"/>
+    <mergeCell ref="E99:L99"/>
+    <mergeCell ref="A115:L115"/>
+    <mergeCell ref="E95:L95"/>
+    <mergeCell ref="A111:L111"/>
+    <mergeCell ref="A117:L117"/>
+    <mergeCell ref="E89:L89"/>
+    <mergeCell ref="E104:L104"/>
+    <mergeCell ref="A114:L114"/>
+    <mergeCell ref="E101:L101"/>
+    <mergeCell ref="E100:L100"/>
+    <mergeCell ref="E91:L91"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="E97:L97"/>
+    <mergeCell ref="A110:L110"/>
+    <mergeCell ref="E102:L102"/>
+    <mergeCell ref="E93:L93"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>